<commit_message>
Update: UI improvements, repair requests, room change workflow, guest management enhancements
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/invoices.xlsx
+++ b/Ma_Nguon/data/excel/invoices.xlsx
@@ -413,701 +413,792 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>invoice_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>contract_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>room_rent</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>electricity_cost</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>water_cost</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>other_fees</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>total_amount</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>due_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>payment_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>payment_method</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>created_at</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>id</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HD202503001</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>INV202510001</t>
+        </is>
+      </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
         <v>2025</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>3500000</v>
       </c>
-      <c r="F2" t="n">
-        <v>157500</v>
-      </c>
       <c r="G2" t="n">
-        <v>45000</v>
+        <v>563500</v>
       </c>
       <c r="H2" t="n">
+        <v>90000</v>
+      </c>
+      <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="n">
-        <v>3702500</v>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="n">
+        <v>4153500</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>paid</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2025-03-10</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2025-03-08</t>
+          <t>2025-10-25</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>2025-10-09T10:00:00</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-03-21T02:51:27.622468</t>
-        </is>
-      </c>
-      <c r="O2" t="n">
-        <v>1</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2025-10-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HD202503003</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>INV202511002</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3" t="n">
         <v>2025</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>3500000</v>
       </c>
-      <c r="F3" t="n">
-        <v>140000</v>
-      </c>
       <c r="G3" t="n">
-        <v>45000</v>
+        <v>388500</v>
       </c>
       <c r="H3" t="n">
+        <v>120000</v>
+      </c>
+      <c r="I3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="n">
-        <v>3685000</v>
-      </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="n">
+        <v>4008500</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>paid</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2025-03-10</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2025-03-09</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>2025-11-06T10:00:00</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-03-21T02:51:27.622477</t>
-        </is>
-      </c>
-      <c r="O3" t="n">
-        <v>3</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2025-11-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>HD202503004</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>INV202512003</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" t="n">
         <v>2025</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>3500000</v>
       </c>
-      <c r="F4" t="n">
-        <v>192500</v>
-      </c>
       <c r="G4" t="n">
-        <v>60000</v>
+        <v>581000</v>
       </c>
       <c r="H4" t="n">
+        <v>195000</v>
+      </c>
+      <c r="I4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="n">
-        <v>3752500</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>unpaid</t>
-        </is>
+      <c r="J4" t="n">
+        <v>4276000</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2025-12-14T10:00:00</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-03-21T02:51:27.622479</t>
-        </is>
-      </c>
-      <c r="O4" t="n">
-        <v>4</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2025-12-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>HD202503005</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>5</v>
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INV202601004</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>2025</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>4500000</v>
+        <v>2026</v>
       </c>
       <c r="F5" t="n">
-        <v>210000</v>
+        <v>3500000</v>
       </c>
       <c r="G5" t="n">
+        <v>469000</v>
+      </c>
+      <c r="H5" t="n">
         <v>75000</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="n">
-        <v>4785000</v>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" t="n">
+        <v>4044000</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>paid</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2025-03-10</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>2026-01-06T10:00:00</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-03-21T02:51:27.622480</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>5</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-01-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>HD202502001</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INV202602005</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="D6" t="n">
-        <v>2025</v>
-      </c>
       <c r="E6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F6" t="n">
         <v>3500000</v>
       </c>
-      <c r="F6" t="n">
-        <v>147000</v>
-      </c>
       <c r="G6" t="n">
-        <v>45000</v>
+        <v>374500</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="I6" t="n">
-        <v>3692000</v>
-      </c>
-      <c r="J6" t="inlineStr">
+        <v>100000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4094500</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>paid</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>2025-02-10</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2025-02-08</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>2026-02-14T10:00:00</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-03-21T02:51:27.622481</t>
-        </is>
-      </c>
-      <c r="O6" t="n">
-        <v>6</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-02-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>HD202502002</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INV202603006</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>2025</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>4000000</v>
+        <v>2026</v>
       </c>
       <c r="F7" t="n">
-        <v>168000</v>
+        <v>3500000</v>
       </c>
       <c r="G7" t="n">
-        <v>60000</v>
+        <v>290500</v>
       </c>
       <c r="H7" t="n">
+        <v>195000</v>
+      </c>
+      <c r="I7" t="n">
         <v>0</v>
       </c>
-      <c r="I7" t="n">
-        <v>4228000</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>unpaid</t>
-        </is>
+      <c r="J7" t="n">
+        <v>3985500</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2025-02-10</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-03-15T10:00:00</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-03-21T02:51:27.622482</t>
-        </is>
-      </c>
-      <c r="O7" t="n">
-        <v>7</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-03-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>HD202603007</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>8</v>
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>INV202510007</t>
+        </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>2026</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
-        <v>12313</v>
+        <v>2025</v>
       </c>
       <c r="F8" t="n">
-        <v>157500</v>
+        <v>3500000</v>
       </c>
       <c r="G8" t="n">
-        <v>75000</v>
+        <v>591500</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>195000</v>
       </c>
       <c r="I8" t="n">
-        <v>244813</v>
-      </c>
-      <c r="J8" t="inlineStr">
+        <v>50000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4336500</v>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>paid</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2025-10-25</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>2025-10-08T10:00:00</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-03-21T18:42:59.300324</t>
-        </is>
-      </c>
-      <c r="O8" t="n">
-        <v>8</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2025-10-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>HD202603008</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>7</v>
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>INV202511008</t>
+        </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>2026</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F9" t="n">
         <v>3500000</v>
       </c>
-      <c r="F9" t="n">
-        <v>157500</v>
-      </c>
       <c r="G9" t="n">
-        <v>45000</v>
+        <v>479500</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>210000</v>
       </c>
       <c r="I9" t="n">
-        <v>3702500</v>
-      </c>
-      <c r="J9" t="inlineStr">
+        <v>50000</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4239500</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>paid</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>2025-11-05T10:00:00</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-03-21T19:22:34.804722</t>
-        </is>
-      </c>
-      <c r="O9" t="n">
-        <v>9</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2025-11-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>HD202603009</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>11</v>
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>INV202512009</t>
+        </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>2026</v>
+        <v>12</v>
       </c>
       <c r="E10" t="n">
-        <v>4000000</v>
+        <v>2025</v>
       </c>
       <c r="F10" t="n">
-        <v>157500</v>
+        <v>3500000</v>
       </c>
       <c r="G10" t="n">
-        <v>75000</v>
+        <v>619500</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>105000</v>
       </c>
       <c r="I10" t="n">
-        <v>4232500</v>
-      </c>
-      <c r="J10" t="inlineStr">
+        <v>100000</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4324500</v>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>paid</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>2025-12-11T10:00:00</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-03-22T04:04:23.676734</t>
-        </is>
-      </c>
-      <c r="O10" t="n">
-        <v>10</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2025-12-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>HD202603010</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3</v>
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>INV202601010</t>
+        </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
         <v>2026</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>3500000</v>
       </c>
-      <c r="F11" t="n">
-        <v>157500</v>
-      </c>
       <c r="G11" t="n">
-        <v>45000</v>
+        <v>430500</v>
       </c>
       <c r="H11" t="n">
+        <v>135000</v>
+      </c>
+      <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="I11" t="n">
-        <v>3702500</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>unpaid</t>
-        </is>
+      <c r="J11" t="n">
+        <v>4065500</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-01-08T10:00:00</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-03-27T00:11:48.636248</t>
-        </is>
-      </c>
-      <c r="O11" t="n">
-        <v>11</v>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-01-01T08:00:00</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>HD202603011</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>INV202602011</t>
+        </is>
+      </c>
       <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="G12" t="n">
+        <v>619500</v>
+      </c>
+      <c r="H12" t="n">
+        <v>150000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4269500</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-02-06T10:00:00</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-02-01T08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>INV202603012</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
         <v>3</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E13" t="n">
         <v>2026</v>
       </c>
-      <c r="E12" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="F12" t="n">
-        <v>157500</v>
-      </c>
-      <c r="G12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>4232500</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>unpaid</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-03-27T00:13:22.181320</t>
-        </is>
-      </c>
-      <c r="O12" t="n">
-        <v>12</v>
+      <c r="F13" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="G13" t="n">
+        <v>448000</v>
+      </c>
+      <c r="H13" t="n">
+        <v>90000</v>
+      </c>
+      <c r="I13" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J13" t="n">
+        <v>4088000</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>transfer</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>2026-03-01T08:00:00</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>